<commit_message>
fix : fixed analysis issues and subject mapping
</commit_message>
<xml_diff>
--- a/data/output/ResultAnalysis.xlsx
+++ b/data/output/ResultAnalysis.xlsx
@@ -692,7 +692,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>086</t>
+          <t>165</t>
         </is>
       </c>
       <c r="O2" s="2" t="n">
@@ -1376,7 +1376,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>041</t>
+          <t>165</t>
         </is>
       </c>
       <c r="O11" s="2" t="n">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>241</t>
+          <t>165</t>
         </is>
       </c>
       <c r="O14" s="2" t="n">
@@ -8748,7 +8748,7 @@
       </c>
       <c r="N108" s="2" t="inlineStr">
         <is>
-          <t>041</t>
+          <t>165</t>
         </is>
       </c>
       <c r="O108" s="2" t="n">
@@ -10040,7 +10040,7 @@
       </c>
       <c r="N125" s="2" t="inlineStr">
         <is>
-          <t>086</t>
+          <t>165</t>
         </is>
       </c>
       <c r="O125" s="2" t="n">
@@ -12511,7 +12511,7 @@
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
     <col width="183" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
     <col width="3" customWidth="1" min="11" max="11"/>
@@ -12897,7 +12897,7 @@
     <row r="32">
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>184</t>
+          <t>English</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -12914,7 +12914,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>184</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -12929,7 +12929,7 @@
     <row r="33">
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -12946,7 +12946,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -12961,24 +12961,24 @@
     <row r="34">
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>041</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>100</v>
+        <v>98.13</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>041</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -12993,24 +12993,24 @@
     <row r="35">
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>086</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>100</v>
+        <v>98.08</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>086</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -13025,7 +13025,7 @@
     <row r="36">
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>087</t>
+          <t>Social Science</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -13042,7 +13042,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>087</t>
+          <t>Social Science</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -13057,14 +13057,14 @@
     <row r="37">
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>Computer Applications</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>0</v>
@@ -13074,7 +13074,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>Computer Applications</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -13089,24 +13089,24 @@
     <row r="38">
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>241</t>
+          <t>Mathematics Basic</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>100</v>
+        <v>97.95999999999999</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>241</t>
+          <t>Mathematics Basic</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">

</xml_diff>